<commit_message>
some changes in FormValidationSteps
</commit_message>
<xml_diff>
--- a/src/main/resources/formData.xlsx
+++ b/src/main/resources/formData.xlsx
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="67" uniqueCount="43">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="79" uniqueCount="44">
   <si>
     <t>First Name</t>
   </si>
@@ -165,6 +165,9 @@
   </si>
   <si>
     <t>CHROME_Result</t>
+  </si>
+  <si>
+    <t>EDGE_Result</t>
   </si>
 </sst>
 </file>
@@ -677,7 +680,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{B324DEF0-A324-4362-B815-B7B052E99BB3}">
-  <dimension ref="A1:Q6"/>
+  <dimension ref="A1:AC6"/>
   <sheetFormatPr defaultRowHeight="14.5"/>
   <cols>
     <col min="5" max="5" bestFit="true" customWidth="true" style="5" width="14.54296875"/>
@@ -725,6 +728,22 @@
       <c r="O1" s="0"/>
       <c r="P1" s="0"/>
       <c r="Q1" s="0"/>
+      <c r="R1" s="0"/>
+      <c r="S1" s="0"/>
+      <c r="T1" s="0"/>
+      <c r="U1" s="0"/>
+      <c r="V1" s="0"/>
+      <c r="W1" s="0"/>
+      <c r="X1" s="0"/>
+      <c r="Y1" s="0"/>
+      <c r="Z1" s="0"/>
+      <c r="AA1" s="0"/>
+      <c r="AB1" t="s" s="0">
+        <v>43</v>
+      </c>
+      <c r="AC1" t="s" s="0">
+        <v>42</v>
+      </c>
     </row>
     <row r="2" spans="1:12" ht="50.5" thickBot="1">
       <c r="A2" s="1">
@@ -763,6 +782,8 @@
       <c r="L2" s="8" t="s">
         <v>40</v>
       </c>
+      <c r="AB2" s="0"/>
+      <c r="AC2" s="0"/>
     </row>
     <row r="3" spans="1:12" ht="50.5" thickBot="1">
       <c r="A3" s="1">
@@ -801,6 +822,8 @@
       <c r="L3" s="2" t="s">
         <v>40</v>
       </c>
+      <c r="AB3" s="0"/>
+      <c r="AC3" s="0"/>
     </row>
     <row r="4" spans="1:12" ht="50.5" thickBot="1">
       <c r="A4" s="1">
@@ -839,6 +862,8 @@
       <c r="L4" s="2" t="s">
         <v>41</v>
       </c>
+      <c r="AB4" s="0"/>
+      <c r="AC4" s="0"/>
     </row>
     <row r="5" spans="1:12" ht="50.5" thickBot="1">
       <c r="A5" s="1">
@@ -877,6 +902,8 @@
       <c r="L5" s="2" t="s">
         <v>41</v>
       </c>
+      <c r="AB5" s="0"/>
+      <c r="AC5" s="0"/>
     </row>
     <row r="6" spans="1:12" ht="63" thickBot="1">
       <c r="A6" s="1">
@@ -913,6 +940,8 @@
       <c r="L6" s="2" t="s">
         <v>41</v>
       </c>
+      <c r="AB6" s="0"/>
+      <c r="AC6" s="0"/>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>

<commit_message>
Full scenario done and dusted
</commit_message>
<xml_diff>
--- a/src/main/resources/formData.xlsx
+++ b/src/main/resources/formData.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://cognizantonline-my.sharepoint.com/personal/2400875_cognizant_com1/Documents/Desktop/LEARN/Cucumber hands-on/Coursera_Cucumber/src/main/resources/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="70" documentId="8_{E2781590-1487-4FF2-8A7A-9B6F8D44F8A7}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{6A5DAD4B-8B96-4607-9B15-1D204876CCDF}"/>
+  <xr:revisionPtr revIDLastSave="71" documentId="8_{E2781590-1487-4FF2-8A7A-9B6F8D44F8A7}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{15D1709B-8C6E-44E5-B48A-5EB75A550A53}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="11500" xr2:uid="{E002FB87-BDFC-460A-A18F-CFA355533938}"/>
   </bookViews>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="79" uniqueCount="44">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="84" uniqueCount="45">
   <si>
     <t>First Name</t>
   </si>
@@ -165,6 +165,9 @@
   </si>
   <si>
     <t>CHROME_Result</t>
+  </si>
+  <si>
+    <t>PASS</t>
   </si>
   <si>
     <t>EDGE_Result</t>
@@ -680,7 +683,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{B324DEF0-A324-4362-B815-B7B052E99BB3}">
-  <dimension ref="A1:AC6"/>
+  <dimension ref="A1:N6"/>
   <sheetFormatPr defaultRowHeight="14.5"/>
   <cols>
     <col min="5" max="5" bestFit="true" customWidth="true" style="5" width="14.54296875"/>
@@ -723,26 +726,11 @@
       <c r="L1" s="13" t="s">
         <v>39</v>
       </c>
-      <c r="M1" s="0"/>
-      <c r="N1" s="0"/>
-      <c r="O1" s="0"/>
-      <c r="P1" s="0"/>
-      <c r="Q1" s="0"/>
-      <c r="R1" s="0"/>
-      <c r="S1" s="0"/>
-      <c r="T1" s="0"/>
-      <c r="U1" s="0"/>
-      <c r="V1" s="0"/>
-      <c r="W1" s="0"/>
-      <c r="X1" s="0"/>
-      <c r="Y1" s="0"/>
-      <c r="Z1" s="0"/>
-      <c r="AA1" s="0"/>
-      <c r="AB1" t="s" s="0">
-        <v>43</v>
-      </c>
-      <c r="AC1" t="s" s="0">
+      <c r="M1" t="s" s="0">
         <v>42</v>
+      </c>
+      <c r="N1" t="s" s="0">
+        <v>44</v>
       </c>
     </row>
     <row r="2" spans="1:12" ht="50.5" thickBot="1">
@@ -782,8 +770,12 @@
       <c r="L2" s="8" t="s">
         <v>40</v>
       </c>
-      <c r="AB2" s="0"/>
-      <c r="AC2" s="0"/>
+      <c r="M2" t="s" s="0">
+        <v>43</v>
+      </c>
+      <c r="N2" t="s" s="0">
+        <v>43</v>
+      </c>
     </row>
     <row r="3" spans="1:12" ht="50.5" thickBot="1">
       <c r="A3" s="1">
@@ -822,8 +814,12 @@
       <c r="L3" s="2" t="s">
         <v>40</v>
       </c>
-      <c r="AB3" s="0"/>
-      <c r="AC3" s="0"/>
+      <c r="M3" t="s" s="0">
+        <v>43</v>
+      </c>
+      <c r="N3" t="s" s="0">
+        <v>43</v>
+      </c>
     </row>
     <row r="4" spans="1:12" ht="50.5" thickBot="1">
       <c r="A4" s="1">
@@ -862,8 +858,12 @@
       <c r="L4" s="2" t="s">
         <v>41</v>
       </c>
-      <c r="AB4" s="0"/>
-      <c r="AC4" s="0"/>
+      <c r="M4" t="s" s="0">
+        <v>43</v>
+      </c>
+      <c r="N4" t="s" s="0">
+        <v>43</v>
+      </c>
     </row>
     <row r="5" spans="1:12" ht="50.5" thickBot="1">
       <c r="A5" s="1">
@@ -902,8 +902,12 @@
       <c r="L5" s="2" t="s">
         <v>41</v>
       </c>
-      <c r="AB5" s="0"/>
-      <c r="AC5" s="0"/>
+      <c r="M5" t="s" s="0">
+        <v>43</v>
+      </c>
+      <c r="N5" t="s" s="0">
+        <v>43</v>
+      </c>
     </row>
     <row r="6" spans="1:12" ht="63" thickBot="1">
       <c r="A6" s="1">
@@ -940,8 +944,12 @@
       <c r="L6" s="2" t="s">
         <v>41</v>
       </c>
-      <c r="AB6" s="0"/>
-      <c r="AC6" s="0"/>
+      <c r="M6" t="s" s="0">
+        <v>43</v>
+      </c>
+      <c r="N6" t="s" s="0">
+        <v>43</v>
+      </c>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>

<commit_message>
Custom Web annotation created
</commit_message>
<xml_diff>
--- a/src/main/resources/formData.xlsx
+++ b/src/main/resources/formData.xlsx
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="143" uniqueCount="45">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="193" uniqueCount="46">
   <si>
     <t>First Name</t>
   </si>
@@ -171,6 +171,9 @@
   </si>
   <si>
     <t>EDGE_Result</t>
+  </si>
+  <si>
+    <t>FAIL</t>
   </si>
 </sst>
 </file>

</xml_diff>